<commit_message>
Workbook Col M (Energy Level filter drop to range 1-3)
</commit_message>
<xml_diff>
--- a/12627043_BhuvanagiriGireesh.xlsx
+++ b/12627043_BhuvanagiriGireesh.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\GiTCloneE\PythonRepo\LPU-PYTHON\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{603101B2-9A18-4A25-B50C-D8AF93091CB4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2D362D7A-0CD6-472E-9526-8CDEBCB69F3F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="22308" windowHeight="13176" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -394,18 +394,18 @@
     <xf numFmtId="0" fontId="6" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="1" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="2" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -706,74 +706,74 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:14" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="10" t="s">
+      <c r="A1" s="12" t="s">
         <v>51</v>
       </c>
-      <c r="B1" s="10"/>
-      <c r="C1" s="10"/>
-      <c r="D1" s="10"/>
-      <c r="E1" s="10"/>
-      <c r="F1" s="10"/>
-      <c r="G1" s="10"/>
-      <c r="H1" s="10"/>
-      <c r="I1" s="10"/>
-      <c r="J1" s="10"/>
-      <c r="K1" s="10"/>
-      <c r="L1" s="10"/>
-      <c r="M1" s="10"/>
-      <c r="N1" s="10"/>
+      <c r="B1" s="12"/>
+      <c r="C1" s="12"/>
+      <c r="D1" s="12"/>
+      <c r="E1" s="12"/>
+      <c r="F1" s="12"/>
+      <c r="G1" s="12"/>
+      <c r="H1" s="12"/>
+      <c r="I1" s="12"/>
+      <c r="J1" s="12"/>
+      <c r="K1" s="12"/>
+      <c r="L1" s="12"/>
+      <c r="M1" s="12"/>
+      <c r="N1" s="12"/>
     </row>
     <row r="2" spans="1:14" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A2" s="2" t="s">
         <v>52</v>
       </c>
-      <c r="B2" s="11" t="s">
+      <c r="B2" s="13" t="s">
         <v>59</v>
       </c>
-      <c r="C2" s="12"/>
-      <c r="D2" s="12"/>
+      <c r="C2" s="14"/>
+      <c r="D2" s="14"/>
       <c r="E2" s="2" t="s">
         <v>53</v>
       </c>
-      <c r="F2" s="13">
+      <c r="F2" s="15">
         <v>12627043</v>
       </c>
-      <c r="G2" s="13"/>
+      <c r="G2" s="15"/>
     </row>
     <row r="3" spans="1:14" ht="21" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="2" t="s">
         <v>54</v>
       </c>
-      <c r="B3" s="11" t="s">
+      <c r="B3" s="13" t="s">
         <v>55</v>
       </c>
-      <c r="C3" s="11"/>
-      <c r="D3" s="11"/>
+      <c r="C3" s="13"/>
+      <c r="D3" s="13"/>
       <c r="E3" s="2" t="s">
         <v>56</v>
       </c>
-      <c r="F3" s="11" t="s">
+      <c r="F3" s="13" t="s">
         <v>57</v>
       </c>
-      <c r="G3" s="11"/>
+      <c r="G3" s="13"/>
     </row>
     <row r="4" spans="1:14" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A4" s="9" t="s">
+      <c r="A4" s="11" t="s">
         <v>58</v>
       </c>
-      <c r="B4" s="9"/>
-      <c r="C4" s="9"/>
-      <c r="D4" s="9"/>
-      <c r="E4" s="9"/>
-      <c r="F4" s="9"/>
-      <c r="G4" s="9"/>
-      <c r="H4" s="9"/>
-      <c r="I4" s="9"/>
-      <c r="J4" s="9"/>
-      <c r="K4" s="9"/>
-      <c r="L4" s="9"/>
-      <c r="M4" s="9"/>
-      <c r="N4" s="9"/>
+      <c r="B4" s="11"/>
+      <c r="C4" s="11"/>
+      <c r="D4" s="11"/>
+      <c r="E4" s="11"/>
+      <c r="F4" s="11"/>
+      <c r="G4" s="11"/>
+      <c r="H4" s="11"/>
+      <c r="I4" s="11"/>
+      <c r="J4" s="11"/>
+      <c r="K4" s="11"/>
+      <c r="L4" s="11"/>
+      <c r="M4" s="11"/>
+      <c r="N4" s="11"/>
     </row>
     <row r="5" spans="1:14" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A5" s="4" t="s">
@@ -849,7 +849,7 @@
         <v>900</v>
       </c>
       <c r="J6" s="6">
-        <f t="shared" ref="J6:J45" si="1">IF(I6="","",1440-I6)</f>
+        <f>IF(I6="","",1440-I6)</f>
         <v>540</v>
       </c>
       <c r="K6" s="1">
@@ -859,7 +859,7 @@
         <v>4</v>
       </c>
       <c r="M6" s="1">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="N6" s="5" t="s">
         <v>14</v>
@@ -895,7 +895,7 @@
         <v>820</v>
       </c>
       <c r="J7" s="6">
-        <f t="shared" si="1"/>
+        <f t="shared" ref="J6:J45" si="1">IF(I7="","",1440-I7)</f>
         <v>620</v>
       </c>
       <c r="K7" s="1">
@@ -905,7 +905,7 @@
         <v>5</v>
       </c>
       <c r="M7" s="1">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="N7" s="5" t="s">
         <v>15</v>
@@ -951,7 +951,7 @@
         <v>4</v>
       </c>
       <c r="M8" s="1">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="N8" s="5" t="s">
         <v>16</v>
@@ -997,7 +997,7 @@
         <v>5</v>
       </c>
       <c r="M9" s="1">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="N9" s="5" t="s">
         <v>17</v>
@@ -1043,7 +1043,7 @@
         <v>4</v>
       </c>
       <c r="M10" s="1">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="N10" s="5" t="s">
         <v>18</v>
@@ -1089,7 +1089,7 @@
         <v>5</v>
       </c>
       <c r="M11" s="1">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="N11" s="5" t="s">
         <v>19</v>
@@ -1135,7 +1135,7 @@
         <v>5</v>
       </c>
       <c r="M12" s="1">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="N12" s="5" t="s">
         <v>14</v>
@@ -1181,7 +1181,7 @@
         <v>5</v>
       </c>
       <c r="M13" s="1">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="N13" s="5" t="s">
         <v>20</v>
@@ -1227,7 +1227,7 @@
         <v>5</v>
       </c>
       <c r="M14" s="1">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="N14" s="5" t="s">
         <v>21</v>
@@ -1273,7 +1273,7 @@
         <v>4</v>
       </c>
       <c r="M15" s="1">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="N15" s="5" t="s">
         <v>22</v>
@@ -1319,7 +1319,7 @@
         <v>4</v>
       </c>
       <c r="M16" s="1">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="N16" s="5" t="s">
         <v>23</v>
@@ -1365,7 +1365,7 @@
         <v>5</v>
       </c>
       <c r="M17" s="1">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="N17" s="5" t="s">
         <v>24</v>
@@ -1411,7 +1411,7 @@
         <v>5</v>
       </c>
       <c r="M18" s="1">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="N18" s="5" t="s">
         <v>25</v>
@@ -1457,7 +1457,7 @@
         <v>4</v>
       </c>
       <c r="M19" s="1">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="N19" s="5" t="s">
         <v>14</v>
@@ -1503,7 +1503,7 @@
         <v>4</v>
       </c>
       <c r="M20" s="1">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="N20" s="5" t="s">
         <v>26</v>
@@ -1549,7 +1549,7 @@
         <v>5</v>
       </c>
       <c r="M21" s="1">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="N21" s="5" t="s">
         <v>27</v>
@@ -1595,7 +1595,7 @@
         <v>5</v>
       </c>
       <c r="M22" s="1">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="N22" s="5" t="s">
         <v>22</v>
@@ -1641,7 +1641,7 @@
         <v>5</v>
       </c>
       <c r="M23" s="1">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="N23" s="5" t="s">
         <v>28</v>
@@ -1687,7 +1687,7 @@
         <v>4</v>
       </c>
       <c r="M24" s="1">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="N24" s="5" t="s">
         <v>29</v>
@@ -1733,7 +1733,7 @@
         <v>4</v>
       </c>
       <c r="M25" s="1">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="N25" s="5" t="s">
         <v>30</v>
@@ -1779,7 +1779,7 @@
         <v>5</v>
       </c>
       <c r="M26" s="1">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="N26" s="5" t="s">
         <v>31</v>
@@ -1825,7 +1825,7 @@
         <v>4</v>
       </c>
       <c r="M27" s="1">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="N27" s="5" t="s">
         <v>32</v>
@@ -1871,7 +1871,7 @@
         <v>4</v>
       </c>
       <c r="M28" s="1">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="N28" s="5" t="s">
         <v>33</v>
@@ -1917,7 +1917,7 @@
         <v>5</v>
       </c>
       <c r="M29" s="1">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="N29" s="5" t="s">
         <v>34</v>
@@ -1963,7 +1963,7 @@
         <v>5</v>
       </c>
       <c r="M30" s="1">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="N30" s="5" t="s">
         <v>35</v>
@@ -2009,7 +2009,7 @@
         <v>4</v>
       </c>
       <c r="M31" s="1">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="N31" s="5" t="s">
         <v>36</v>
@@ -2055,7 +2055,7 @@
         <v>4</v>
       </c>
       <c r="M32" s="1">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="N32" s="5" t="s">
         <v>37</v>
@@ -2101,7 +2101,7 @@
         <v>4</v>
       </c>
       <c r="M33" s="1">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="N33" s="5" t="s">
         <v>38</v>
@@ -2147,7 +2147,7 @@
         <v>5</v>
       </c>
       <c r="M34" s="1">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="N34" s="5" t="s">
         <v>39</v>
@@ -2193,7 +2193,7 @@
         <v>5</v>
       </c>
       <c r="M35" s="1">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="N35" s="5" t="s">
         <v>40</v>
@@ -2239,7 +2239,7 @@
         <v>5</v>
       </c>
       <c r="M36" s="1">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="N36" s="5" t="s">
         <v>41</v>
@@ -2285,7 +2285,7 @@
         <v>5</v>
       </c>
       <c r="M37" s="1">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="N37" s="5" t="s">
         <v>42</v>
@@ -2331,7 +2331,7 @@
         <v>4</v>
       </c>
       <c r="M38" s="1">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="N38" s="5" t="s">
         <v>43</v>
@@ -2377,7 +2377,7 @@
         <v>4</v>
       </c>
       <c r="M39" s="1">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="N39" s="5" t="s">
         <v>44</v>
@@ -2423,7 +2423,7 @@
         <v>5</v>
       </c>
       <c r="M40" s="1">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="N40" s="5" t="s">
         <v>45</v>
@@ -2469,7 +2469,7 @@
         <v>4</v>
       </c>
       <c r="M41" s="1">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="N41" s="5" t="s">
         <v>46</v>
@@ -2515,7 +2515,7 @@
         <v>4</v>
       </c>
       <c r="M42" s="1">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="N42" s="5" t="s">
         <v>47</v>
@@ -2561,7 +2561,7 @@
         <v>5</v>
       </c>
       <c r="M43" s="1">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="N43" s="5" t="s">
         <v>48</v>
@@ -2607,7 +2607,7 @@
         <v>5</v>
       </c>
       <c r="M44" s="1">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="N44" s="5" t="s">
         <v>49</v>
@@ -2653,7 +2653,7 @@
         <v>5</v>
       </c>
       <c r="M45" s="1">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="N45" s="5" t="s">
         <v>50</v>
@@ -2709,43 +2709,43 @@
       </c>
       <c r="M46" s="8">
         <f>AVERAGE(M6:M45)</f>
-        <v>4.7750000000000004</v>
+        <v>2.625</v>
       </c>
     </row>
     <row r="47" spans="1:14" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A47" s="14" t="s">
+      <c r="A47" s="9" t="s">
         <v>61</v>
       </c>
-      <c r="B47" s="15">
+      <c r="B47" s="10">
         <f>AVERAGE(B6:B45)</f>
         <v>402</v>
       </c>
-      <c r="C47" s="15">
+      <c r="C47" s="10">
         <f t="shared" ref="C47:J47" si="3">AVERAGE(C6:C45)</f>
         <v>27.5</v>
       </c>
-      <c r="D47" s="15">
+      <c r="D47" s="10">
         <f t="shared" si="3"/>
         <v>99</v>
       </c>
-      <c r="E47" s="15">
+      <c r="E47" s="10">
         <f t="shared" si="3"/>
         <v>38.25</v>
       </c>
-      <c r="F47" s="15">
+      <c r="F47" s="10">
         <f t="shared" si="3"/>
         <v>216</v>
       </c>
-      <c r="G47" s="15">
+      <c r="G47" s="10">
         <f t="shared" si="3"/>
         <v>3.6</v>
       </c>
-      <c r="H47" s="15">
+      <c r="H47" s="10">
         <f t="shared" si="3"/>
         <v>82.75</v>
       </c>
-      <c r="I47" s="15"/>
-      <c r="J47" s="15">
+      <c r="I47" s="10"/>
+      <c r="J47" s="10">
         <f t="shared" si="3"/>
         <v>574.5</v>
       </c>

</xml_diff>